<commit_message>
Se termino de diseñar la version 2 del nodo ambiente, ahora se va a diseñar el case3d para que contenga al mismo
</commit_message>
<xml_diff>
--- a/workspace/systemMonitorLab/hardware/NodoAmbienteSMN/NodoV2/pcb_build_resources/listaComponentesCompra.xlsx
+++ b/workspace/systemMonitorLab/hardware/NodoAmbienteSMN/NodoV2/pcb_build_resources/listaComponentesCompra.xlsx
@@ -1,27 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\esp\ESP8266_RTOS_SDK\workspace\systemMonitorLab\hardware\NodoAmbienteSMN\NodoV2\pcb_build_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4720F24-BB23-4B76-BBD3-928A9D32DC9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11490"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="listaComponentesCompra" sheetId="1" r:id="rId1"/>
     <sheet name="BOM" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="152511"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="75">
   <si>
     <t>Reference</t>
   </si>
@@ -247,12 +260,19 @@
   </si>
   <si>
     <t>https://www.sycelectronica.com.ar/articulo.php?codigo=CR1206-47</t>
+  </si>
+  <si>
+    <t>https://www.sycelectronica.com.ar/articulo.php?codigo=FCG10C</t>
+  </si>
+  <si>
+    <t>FCG10C
+CABLE PLANO 10 VIAS COLOR (18 metros)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -405,7 +425,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -618,6 +638,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -798,7 +824,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -835,6 +861,9 @@
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -855,7 +884,7 @@
     <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
     <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
     <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Buena" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
     <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
@@ -1156,7 +1185,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1202,7 +1231,7 @@
         <f>A2*6</f>
         <v>36</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="18" t="s">
         <v>52</v>
       </c>
       <c r="D2" s="7" t="s">
@@ -1225,7 +1254,7 @@
         <f t="shared" ref="B3:B20" si="0">A3*6</f>
         <v>0</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="18" t="s">
         <v>51</v>
       </c>
       <c r="D3" s="7" t="s">
@@ -1250,7 +1279,7 @@
         <f>A4*6</f>
         <v>36</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="18" t="s">
         <v>53</v>
       </c>
       <c r="D4" s="7" t="s">
@@ -1275,7 +1304,7 @@
         <f>A5*6</f>
         <v>6</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="18" t="s">
         <v>57</v>
       </c>
       <c r="D5" s="7" t="s">
@@ -1323,7 +1352,7 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="18" t="s">
         <v>64</v>
       </c>
       <c r="D7" s="7" t="s">
@@ -1348,7 +1377,7 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="18" t="s">
         <v>65</v>
       </c>
       <c r="D8" s="7" t="s">
@@ -1398,7 +1427,7 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="18" t="s">
         <v>69</v>
       </c>
       <c r="D10" s="7" t="s">
@@ -1423,7 +1452,7 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="18" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="7" t="s">
@@ -1440,14 +1469,20 @@
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
+        <v>3</v>
+      </c>
       <c r="B12" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="6"/>
+        <v>18</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>73</v>
+      </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6">
         <f t="shared" si="1"/>
@@ -1586,24 +1621,25 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1"/>
-    <hyperlink ref="D2" r:id="rId2"/>
-    <hyperlink ref="D4" r:id="rId3"/>
-    <hyperlink ref="D5" r:id="rId4"/>
-    <hyperlink ref="D6" r:id="rId5"/>
-    <hyperlink ref="D7" r:id="rId6"/>
-    <hyperlink ref="D8" r:id="rId7"/>
-    <hyperlink ref="D9" r:id="rId8"/>
-    <hyperlink ref="D10" r:id="rId9"/>
-    <hyperlink ref="D11" r:id="rId10"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId12"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2078,13 +2114,13 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E10" r:id="rId1"/>
-    <hyperlink ref="E9" r:id="rId2"/>
-    <hyperlink ref="E8" r:id="rId3"/>
-    <hyperlink ref="E6" r:id="rId4"/>
-    <hyperlink ref="E5" r:id="rId5"/>
-    <hyperlink ref="E4" r:id="rId6"/>
-    <hyperlink ref="H11" r:id="rId7" location="cha_BJTs"/>
+    <hyperlink ref="E10" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="E9" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="E8" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="E6" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="E5" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="E4" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+    <hyperlink ref="H11" r:id="rId7" location="cha_BJTs" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>